<commit_message>
Actualizacion de data de deployment en USA
</commit_message>
<xml_diff>
--- a/p6_deployment/data/usa/data_preparation/df_etiquetas_actualizado.xlsx
+++ b/p6_deployment/data/usa/data_preparation/df_etiquetas_actualizado.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1377"/>
+  <dimension ref="A1:C1418"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21159,6 +21159,625 @@
         <v>170</v>
       </c>
     </row>
+    <row r="1378">
+      <c r="A1378" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B1378" t="inlineStr">
+        <is>
+          <t>Sd7snoa0</t>
+        </is>
+      </c>
+      <c r="C1378" t="n">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="1379">
+      <c r="A1379" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B1379" t="inlineStr">
+        <is>
+          <t>GzULyFoh</t>
+        </is>
+      </c>
+      <c r="C1379" t="n">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="1380">
+      <c r="A1380" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B1380" t="inlineStr">
+        <is>
+          <t>dp6AQn9c</t>
+        </is>
+      </c>
+      <c r="C1380" t="n">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="1381">
+      <c r="A1381" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B1381" t="inlineStr">
+        <is>
+          <t>l6eEjGlO</t>
+        </is>
+      </c>
+      <c r="C1381" t="n">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="1382">
+      <c r="A1382" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B1382" t="inlineStr">
+        <is>
+          <t>86yPt28f</t>
+        </is>
+      </c>
+      <c r="C1382" t="n">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="1383">
+      <c r="A1383" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B1383" t="inlineStr">
+        <is>
+          <t>GzULyFoh</t>
+        </is>
+      </c>
+      <c r="C1383" t="n">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="1384">
+      <c r="A1384" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B1384" t="inlineStr">
+        <is>
+          <t>z9ZXDy6o</t>
+        </is>
+      </c>
+      <c r="C1384" t="n">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="1385">
+      <c r="A1385" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B1385" t="inlineStr">
+        <is>
+          <t>6BusaLE3</t>
+        </is>
+      </c>
+      <c r="C1385" t="n">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="1386">
+      <c r="A1386" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B1386" t="inlineStr">
+        <is>
+          <t>roEEsq76</t>
+        </is>
+      </c>
+      <c r="C1386" t="n">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="1387">
+      <c r="A1387" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B1387" t="inlineStr">
+        <is>
+          <t>6BusaLE3</t>
+        </is>
+      </c>
+      <c r="C1387" t="n">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="1388">
+      <c r="A1388" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B1388" t="inlineStr">
+        <is>
+          <t>K4zRMgTN</t>
+        </is>
+      </c>
+      <c r="C1388" t="n">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="1389">
+      <c r="A1389" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B1389" t="inlineStr">
+        <is>
+          <t>6gpXy3vi</t>
+        </is>
+      </c>
+      <c r="C1389" t="n">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="1390">
+      <c r="A1390" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B1390" t="inlineStr">
+        <is>
+          <t>6gpXy3vi</t>
+        </is>
+      </c>
+      <c r="C1390" t="n">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="1391">
+      <c r="A1391" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B1391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ndiaye a 
+  usa </t>
+        </is>
+      </c>
+      <c r="C1391" t="n">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="1392">
+      <c r="A1392" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B1392" t="inlineStr">
+        <is>
+          <t>bFuhdIb3</t>
+        </is>
+      </c>
+      <c r="C1392" t="n">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="1393">
+      <c r="A1393" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B1393" t="inlineStr">
+        <is>
+          <t>WWvwigh8</t>
+        </is>
+      </c>
+      <c r="C1393" t="n">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="1394">
+      <c r="A1394" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B1394" t="inlineStr">
+        <is>
+          <t>lAVQ9RGh</t>
+        </is>
+      </c>
+      <c r="C1394" t="n">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="1395">
+      <c r="A1395" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B1395" t="inlineStr">
+        <is>
+          <t>UFWZoX9L</t>
+        </is>
+      </c>
+      <c r="C1395" t="n">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="1396">
+      <c r="A1396" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B1396" t="inlineStr">
+        <is>
+          <t>jBBpU7Y0</t>
+        </is>
+      </c>
+      <c r="C1396" t="n">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="1397">
+      <c r="A1397" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B1397" t="inlineStr">
+        <is>
+          <t>MFwJSk8d</t>
+        </is>
+      </c>
+      <c r="C1397" t="n">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="1398">
+      <c r="A1398" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B1398" t="inlineStr">
+        <is>
+          <t>xA45kovo</t>
+        </is>
+      </c>
+      <c r="C1398" t="n">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="1399">
+      <c r="A1399" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B1399" t="inlineStr">
+        <is>
+          <t>6LuGZiZI</t>
+        </is>
+      </c>
+      <c r="C1399" t="n">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="1400">
+      <c r="A1400" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B1400" t="inlineStr">
+        <is>
+          <t>nJ01AhXP</t>
+        </is>
+      </c>
+      <c r="C1400" t="n">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="1401">
+      <c r="A1401" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B1401" t="inlineStr">
+        <is>
+          <t>2PIEeC7j</t>
+        </is>
+      </c>
+      <c r="C1401" t="n">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="1402">
+      <c r="A1402" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B1402" t="inlineStr">
+        <is>
+          <t>WSL0wFD4</t>
+        </is>
+      </c>
+      <c r="C1402" t="n">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="1403">
+      <c r="A1403" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B1403" t="inlineStr">
+        <is>
+          <t>EgT3xN3S</t>
+        </is>
+      </c>
+      <c r="C1403" t="n">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="1404">
+      <c r="A1404" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B1404" t="inlineStr">
+        <is>
+          <t>bFuhdIb3</t>
+        </is>
+      </c>
+      <c r="C1404" t="n">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="1405">
+      <c r="A1405" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B1405" t="inlineStr">
+        <is>
+          <t>EqKWmJfM</t>
+        </is>
+      </c>
+      <c r="C1405" t="n">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="1406">
+      <c r="A1406" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B1406" t="inlineStr">
+        <is>
+          <t>UL7r7duf</t>
+        </is>
+      </c>
+      <c r="C1406" t="n">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="1407">
+      <c r="A1407" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B1407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">touchan r 
+  usa </t>
+        </is>
+      </c>
+      <c r="C1407" t="n">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="1408">
+      <c r="A1408" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B1408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">montero r 
+  cos </t>
+        </is>
+      </c>
+      <c r="C1408" t="n">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="1409">
+      <c r="A1409" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B1409" t="inlineStr">
+        <is>
+          <t>URfp4iBR</t>
+        </is>
+      </c>
+      <c r="C1409" t="n">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="1410">
+      <c r="A1410" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B1410" t="inlineStr">
+        <is>
+          <t>txm4BKVR</t>
+        </is>
+      </c>
+      <c r="C1410" t="n">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="1411">
+      <c r="A1411" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B1411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">snyder t 
+  usa </t>
+        </is>
+      </c>
+      <c r="C1411" t="n">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="1412">
+      <c r="A1412" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B1412" t="inlineStr">
+        <is>
+          <t>CfE5JcGF</t>
+        </is>
+      </c>
+      <c r="C1412" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="1413">
+      <c r="A1413" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B1413" t="inlineStr">
+        <is>
+          <t>KtuTuMN0</t>
+        </is>
+      </c>
+      <c r="C1413" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="1414">
+      <c r="A1414" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B1414" t="inlineStr">
+        <is>
+          <t>K4FYmLD9</t>
+        </is>
+      </c>
+      <c r="C1414" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="1415">
+      <c r="A1415" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B1415" t="inlineStr">
+        <is>
+          <t>rJ9D8rzj</t>
+        </is>
+      </c>
+      <c r="C1415" t="n">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="1416">
+      <c r="A1416" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B1416" t="inlineStr">
+        <is>
+          <t>rJ9D8rzj</t>
+        </is>
+      </c>
+      <c r="C1416" t="n">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="1417">
+      <c r="A1417" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B1417" t="inlineStr">
+        <is>
+          <t>pKAODsPO</t>
+        </is>
+      </c>
+      <c r="C1417" t="n">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="1418">
+      <c r="A1418" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B1418" t="inlineStr">
+        <is>
+          <t>tOpyQa24</t>
+        </is>
+      </c>
+      <c r="C1418" t="n">
+        <v>197</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>